<commit_message>
docs: Care+ banner restyle is International only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/international/International_Registration_Report.xlsx
+++ b/docs/international/International_Registration_Report.xlsx
@@ -17,7 +17,7 @@
     <sheet name="Run &amp; Open Items" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$4:$B$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$4:$B$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fields'!$A$4:$E$39</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Errors'!$A$4:$D$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'APIs'!$A$4:$D$14</definedName>
@@ -506,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -803,12 +803,24 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Unchanged, except the Care+ banner restyled to match the screens</t>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Decision · Care+ banner</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>International only: light-peach banner with an orange dashed border, as in the screens</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:B27"/>
+  <autoFilter ref="A4:B28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3776,7 +3788,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Shared pieces exported, tabs clickable, Care+ banner restyled</t>
+          <t>Shared pieces exported, tabs clickable (form unchanged)</t>
         </is>
       </c>
     </row>

</xml_diff>